<commit_message>
Add sample monthly bookkeeping pack and monthly report
Fictional business, labelled as sample data. Workbook recalculates from its inputs; the report is a two-page PDF of its Monthly Report sheet at full width.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_017mRBpKsgGkNpLR25J7Ae3C
</commit_message>
<xml_diff>
--- a/templates/CayTech-Sample-Monthly-Bookkeeping-Pack.xlsx
+++ b/templates/CayTech-Sample-Monthly-Bookkeeping-Pack.xlsx
@@ -523,7 +523,7 @@
     <t xml:space="preserve">What is included</t>
   </si>
   <si>
-    <t xml:space="preserve">Monthly rent roll with arrears follow-up list; bar stock and takings check; expense log; cash reconciliation to your bank / mobile money statements; one-page monthly report with plain-language findings.</t>
+    <t xml:space="preserve">Monthly rent roll with arrears follow-up list; bar stock and takings check; expense log; cash reconciliation to your bank / mobile money statements; monthly report with plain-language findings.</t>
   </si>
   <si>
     <t xml:space="preserve">What is not included</t>
@@ -1508,8 +1508,8 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2077,13 +2077,13 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.5" right="0.5" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;8 SAMPLE DATA - FICTIONAL</oddHeader>
     <oddFooter>&amp;L&amp;8 Prepared by Caristo Mulenga | CayTech Digital Solutions | WhatsApp +260 963 149 074&amp;R&amp;8 Page &amp;P</oddFooter>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="41" man="true" max="16383" min="0"/>
+    <brk id="57" man="true" max="16383" min="0"/>
   </rowBreaks>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>